<commit_message>
Run v2 purchase suite with 2 parallel devices; expand purchase-data matrix
- testng-parallel-purchase.xml: data-provider-thread-count 1 -> 2, so both
  configured BrowserStack devices run concurrently instead of sequentially.
  Verified clean on both Google Pixel 8 and Samsung Galaxy S24 (Tests run: 2,
  Failures: 0) after the prior session's WEBVIEW/splash-screen fixes.

- TestData/PurchaseData-v2.xlsx: added 4 more payment-method rows (Wallet,
  Cash on Delivery, Google Pay, Credit/Debit Card) alongside the existing Net
  Banking row. The sheet has no Execute column, so PurchaseDataReader runs
  every non-empty row unconditionally - this was previously a single row,
  which is why every prior v2 purchase run only ever exercised Net Banking.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ma7mHY9Sj29Ht4gaAHtkdS
</commit_message>
<xml_diff>
--- a/TestData/PurchaseData-v2.xlsx
+++ b/TestData/PurchaseData-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E24C68-F72C-40F1-BB25-91618527B4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F9C000-459A-4BF1-A7EB-21DB224145EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="30">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -621,61 +621,144 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="B2" s="5"/>
       <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="11" t="s">
-        <v>24</v>
+      <c r="D2" s="7"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="12" t="s">
+        <v>27</v>
       </c>
       <c r="K2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="11"/>
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="12"/>
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="K6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I12" s="8"/>

</xml_diff>